<commit_message>
Genericize persona company to Contoso Investment Bank Berhad
Replace all narrative Kenanga / KIBB references with Contoso across the
site, the README, and the regenerated data files. File names retained
(01_KIBB_*.xlsx etc.) since they are committed assets. Site title and
sidebar branding now read 'Contoso Investment Bank Berhad'.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/01_KIBB_SegmentPnL.xlsx
+++ b/files/01_KIBB_SegmentPnL.xlsx
@@ -531,7 +531,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kenanga Investment Bank Berhad - Group Monthly Operating Cost (RM '000)</t>
+          <t>Contoso Investment Bank Berhad - Group Monthly Operating Cost (RM '000)</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>CEO, Kenanga Investors</t>
+          <t>CEO, Contoso Investors</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1640,7 +1640,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KIBB Segment Revenue (RM '000) - FY2026 YTD</t>
+          <t>Contoso Segment Revenue (RM '000) - FY2026 YTD</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KIBB Group KPIs - FY2026 YTD</t>
+          <t>Contoso Group KPIs - FY2026 YTD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix data realism: remove brand leaks, tie BRC numbers to workbook, reframe as FY2025 year-end
- Vendor contract: replace 2 KENANGA INVESTMENT BANK BERHAD references and Kenanga company numbers with Contoso fictionals
- BRC transcript: drop Subramaniam surname (persona is first-name only), replace KDi GO and Rakuten product names with generics, tighten revenue/cost variance numbers (5.6% / 12.9%) to match workbook, reflect AWM as red (not amber) given 11.5% breach
- Workbook: relabel FY2026 -> FY2025 (Final Audited) so 12 months of Jan-Dec data is internally consistent with the 27 March 2026 BRC review timing
- index.html: reframe Q1 BRC narrative to FY2025 year-end where required, switch Analyst Agent prompt to use cost-vs-budget data the workbook actually contains

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/01_KIBB_SegmentPnL.xlsx
+++ b/files/01_KIBB_SegmentPnL.xlsx
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FY2026 - Source: Group Finance - Confidential: Board Risk Committee</t>
+          <t>FY2025 (Final Audited) - Source: Group Finance - Confidential: Board Risk Committee</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Contoso Segment Revenue (RM '000) - FY2026 YTD</t>
+          <t>Contoso Segment Revenue (RM '000) - FY2025 Full Year</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Contoso Group KPIs - FY2026 YTD</t>
+          <t>Contoso Group KPIs - FY2025 Full Year</t>
         </is>
       </c>
     </row>
@@ -1912,12 +1912,12 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>FY2026 YTD</t>
+          <t>FY2025 Actual</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>FY2026 Budget / Threshold</t>
+          <t>FY2025 Budget / Threshold</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Slipped from 25.3% (FY24) - Rakuten platform stability</t>
+          <t>Slipped from 25.3% (FY24) - retail trading platform stability issues</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>KDi GO uptake slower than plan</t>
+          <t>Digital wealth platform uptake slower than plan</t>
         </is>
       </c>
     </row>

</xml_diff>